<commit_message>
Agrega hoja Tarifa y Margen: tarifa por envio para 30% de margen (operador logistico)
</commit_message>
<xml_diff>
--- a/Evaluacion_Flota_vs_Courier.xlsx
+++ b/Evaluacion_Flota_vs_Courier.xlsx
@@ -5,7 +5,8 @@
     <sheet name="Supuestos" sheetId="1" r:id="rId1"/>
     <sheet name="Escenarios" sheetId="2" r:id="rId2"/>
     <sheet name="Electrica vs Courier" sheetId="3" r:id="rId3"/>
-    <sheet name="Proyeccion 3 anos" sheetId="4" r:id="rId4"/>
+    <sheet name="Tarifa y Margen" sheetId="4" r:id="rId4"/>
+    <sheet name="Proyeccion 3 anos" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,6 +487,33 @@
         <v>0.04</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA / MARGEN (operador logistico)</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen objetivo (% sobre venta)</t>
+        </is>
+      </c>
+      <c r="B41" s="5">
+        <v>0.3</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1092,6 +1120,319 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA COMO OPERADOR LOGISTICO  (margen objetivo sobre venta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa que debes cobrar para cubrir costos y dejar el margen de Supuestos!B41. Compara contra el courier ($/envio actual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen objetivo:</t>
+        </is>
+      </c>
+      <c r="B3" s="10">
+        <f>Supuestos!$B$41</f>
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concepto</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flota Electrica</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flota Petrolera</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Courier (ref.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo total / mes</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+(Supuestos!$B$10*Supuestos!$B$24)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
+        <v>29811000.0</v>
+      </c>
+      <c r="C6" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
+        <v>29701000.0</v>
+      </c>
+      <c r="D6" s="8">
+        <f>Supuestos!$B$8*Supuestos!$B$5</f>
+        <v>44700000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo por envio</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>B6/Supuestos!$B$5</f>
+        <v>1987.4</v>
+      </c>
+      <c r="C7" s="8">
+        <f>C6/Supuestos!$B$5</f>
+        <v>1980.0666666666666</v>
+      </c>
+      <c r="D7" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA por envio (con margen)</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>B7/(1-Supuestos!$B$41)</f>
+        <v>2839.1428571428573</v>
+      </c>
+      <c r="C8" s="9">
+        <f>C7/(1-Supuestos!$B$41)</f>
+        <v>2828.666666666667</v>
+      </c>
+      <c r="D8" s="9">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facturacion / mes (a esa tarifa)</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>B6/(1-Supuestos!$B$41)</f>
+        <v>42587142.85714286</v>
+      </c>
+      <c r="C9" s="8">
+        <f>C6/(1-Supuestos!$B$41)</f>
+        <v>42430000.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen $ / mes</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>B9-B6</f>
+        <v>12776142.857142858</v>
+      </c>
+      <c r="C10" s="8">
+        <f>C9-C6</f>
+        <v>12729000.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen $ / ano</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>B10*12</f>
+        <v>153313714.2857143</v>
+      </c>
+      <c r="C11" s="9">
+        <f>C10*12</f>
+        <v>152748000.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa vs courier (ahorro/envio)</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>Supuestos!$B$8-B8</f>
+        <v>140.85714285714266</v>
+      </c>
+      <c r="C12" s="9">
+        <f>Supuestos!$B$8-C8</f>
+        <v>151.33333333333303</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa % bajo el courier</t>
+        </is>
+      </c>
+      <c r="B13" s="10">
+        <f>(Supuestos!$B$8-B8)/Supuestos!$B$8</f>
+        <v>0.04726749760306801</v>
+      </c>
+      <c r="C13" s="10">
+        <f>(Supuestos!$B$8-C8)/Supuestos!$B$8</f>
+        <v>0.050782997762863435</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA POR ENVIO SEGUN TAMANO DE FLOTA (con margen objetivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moviles (N)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa Elec.</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa Pet.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Courier (ref.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11">
+        <v>10</v>
+      </c>
+      <c r="B17" s="8">
+        <f>(($A17*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A17*Supuestos!$B$24)+($A17*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A17*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A17*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3692.857142857143</v>
+      </c>
+      <c r="C17" s="8">
+        <f>(($A17*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A17*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A17*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A17*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3595.2380952380954</v>
+      </c>
+      <c r="D17" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11">
+        <v>9</v>
+      </c>
+      <c r="B18" s="8">
+        <f>(($A18*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A18*Supuestos!$B$24)+($A18*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A18*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A18*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3408.2857142857147</v>
+      </c>
+      <c r="C18" s="8">
+        <f>(($A18*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A18*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A18*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A18*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3339.7142857142862</v>
+      </c>
+      <c r="D18" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <v>8</v>
+      </c>
+      <c r="B19" s="8">
+        <f>(($A19*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A19*Supuestos!$B$24)+($A19*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A19*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A19*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3123.714285714286</v>
+      </c>
+      <c r="C19" s="8">
+        <f>(($A19*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A19*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A19*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A19*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3084.1904761904766</v>
+      </c>
+      <c r="D19" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11">
+        <v>7</v>
+      </c>
+      <c r="B20" s="8">
+        <f>(($A20*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A20*Supuestos!$B$24)+($A20*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A20*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A20*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2839.1428571428573</v>
+      </c>
+      <c r="C20" s="8">
+        <f>(($A20*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A20*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A20*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A20*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2828.666666666667</v>
+      </c>
+      <c r="D20" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11">
+        <v>6</v>
+      </c>
+      <c r="B21" s="8">
+        <f>(($A21*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A21*Supuestos!$B$24)+($A21*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A21*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A21*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2554.571428571429</v>
+      </c>
+      <c r="C21" s="8">
+        <f>(($A21*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A21*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A21*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A21*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2573.1428571428573</v>
+      </c>
+      <c r="D21" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota: margen sobre venta -&gt; tarifa = costo / (1 - margen). Si la tarifa es menor al courier, eres competitivo Y rentable.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>

</xml_diff>

<commit_message>
Agrega hoja Resumen Ejecutivo (primera) con cifras vivas y narrativa para directorio
</commit_message>
<xml_diff>
--- a/Evaluacion_Flota_vs_Courier.xlsx
+++ b/Evaluacion_Flota_vs_Courier.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Supuestos" sheetId="1" r:id="rId1"/>
-    <sheet name="Escenarios" sheetId="2" r:id="rId2"/>
-    <sheet name="Electrica vs Courier" sheetId="3" r:id="rId3"/>
-    <sheet name="Tarifa y Margen" sheetId="4" r:id="rId4"/>
-    <sheet name="Proyeccion 3 anos" sheetId="5" r:id="rId5"/>
+    <sheet name="Resumen Ejecutivo" sheetId="1" r:id="rId1"/>
+    <sheet name="Supuestos" sheetId="2" r:id="rId2"/>
+    <sheet name="Escenarios" sheetId="3" r:id="rId3"/>
+    <sheet name="Electrica vs Courier" sheetId="4" r:id="rId4"/>
+    <sheet name="Tarifa y Margen" sheetId="5" r:id="rId5"/>
+    <sheet name="Proyeccion 3 anos" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -96,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -113,6 +114,9 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -123,6 +127,298 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RESUMEN EJECUTIVO  -  Internalizacion de Ultima Milla</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluacion: flota propia electrica vs. courier actual  (CAV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CIFRAS CLAVE  (escenario base: flota electrica)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Indicador</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Envios por mes</t>
+        </is>
+      </c>
+      <c r="B6" s="11">
+        <f>Supuestos!$B$5</f>
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N de moviles (escenario base)</t>
+        </is>
+      </c>
+      <c r="B7" s="11">
+        <f>Supuestos!$B$10</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo courier actual (por envio)</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo courier (por mes)</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>Supuestos!$B$8*Supuestos!$B$5</f>
+        <v>44700000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo flota electrica (por mes)</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+(Supuestos!$B$10*Supuestos!$B$24)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
+        <v>29811000.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo flota electrica (por envio)</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>B9/Supuestos!$B$5</f>
+        <v>1987.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahorro mensual vs courier</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>B8-B9</f>
+        <v>14889000.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahorro ANUAL vs courier</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>(B8-B9)*12</f>
+        <v>178668000.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reduccion de costo</t>
+        </is>
+      </c>
+      <c r="B14" s="10">
+        <f>(B8-B9)/B8</f>
+        <v>0.33308724832214764</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utilizacion de capacidad</t>
+        </is>
+      </c>
+      <c r="B15" s="10">
+        <f>Supuestos!$B$5/(Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10)</f>
+        <v>0.8116883116883117</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto de equilibrio (envios/mes)</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
+        <f>B9/Supuestos!$B$8</f>
+        <v>10003.691275167785</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa con margen objetivo (por envio)</t>
+        </is>
+      </c>
+      <c r="B17" s="9">
+        <f>B10/(1-Supuestos!$B$41)</f>
+        <v>2839.1428571428573</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen ANUAL como operador logistico</t>
+        </is>
+      </c>
+      <c r="B18" s="9">
+        <f>(B9/(1-Supuestos!$B$41)-B9)*12</f>
+        <v>153313714.2857143</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LECTURA PARA EL DIRECTORIO</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Internalizar la ultima milla reduce el costo de despacho ~33%: de $2.980 a ~$1.987 por envio, con un ahorro de ~$179 millones al ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. La flota actual estaria sobredimensionada: con capacidad de 120 puntos por ruta, bastan 6-7 moviles para cubrir los 15.000 envios. Con 7 operamos al 81% y queda holgura para crecer sin sumar vehiculos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Electrico vs petrolero: hoy practicamente empatan en costo. En 3 anos, con el diesel subiendo mas rapido, el electrico pasa a ser mas barato desde el Ano 2 y amplia su ventaja (mas sostenibilidad e imagen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. Como operador logistico podemos ser mas baratos Y rentables: una tarifa con 30% de margen (~$2.840/envio) sigue ~5% bajo el courier actual, con un margen potencial de ~$153 millones al ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RECOMENDACION</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avanzar hacia una flota propia de 7 moviles electricos (mejor balance entre ahorro y holgura operacional). Como alternativa de menor riesgo inicial, evaluar un modelo hibrido: flota propia para la base estable + courier para los peaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RIESGOS Y CONDICIONES</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Sobrekilometraje: con 7 moviles cada uno recorre ~4.300 km/mes (contrato 3.000). Ya esta en el costo; conviene negociar el limite de km.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Costo fijo vs variable: la flota conviene mientras el volumen supere ~10.000 envios/mes; bajo ese nivel el courier vuelve a ser preferible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Gestion de personas: se asumen 14 colaboradores (conductores + peonetas) con su administracion y relacion laboral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota: todas las cifras se recalculan al editar la hoja "Supuestos" (celdas amarillas). Valores de referencia a confirmar con cotizaciones formales.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
@@ -518,7 +814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -817,306 +1113,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EVALUACION: FLOTA ELECTRICA vs COURIER</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Moviles del escenario base (editar en Supuestos!B10):</t>
-        </is>
-      </c>
-      <c r="B2" s="11">
-        <f>Supuestos!$B$10</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Concepto</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Courier</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Flota Electrica</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diferencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Costo total / mes</t>
-        </is>
-      </c>
-      <c r="B5" s="8">
-        <f>Supuestos!$B$8*Supuestos!$B$5</f>
-        <v>44700000</v>
-      </c>
-      <c r="C5" s="8">
-        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+(Supuestos!$B$10*Supuestos!$B$24)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
-        <v>29811000.0</v>
-      </c>
-      <c r="D5" s="9">
-        <f>C5-B5</f>
-        <v>-14889000.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Costo por envio</t>
-        </is>
-      </c>
-      <c r="B6" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
-      </c>
-      <c r="C6" s="8">
-        <f>C5/Supuestos!$B$5</f>
-        <v>1987.4</v>
-      </c>
-      <c r="D6" s="9">
-        <f>C6-B6</f>
-        <v>-992.5999999999999</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Costo total / ano</t>
-        </is>
-      </c>
-      <c r="B7" s="8">
-        <f>B5*12</f>
-        <v>536400000</v>
-      </c>
-      <c r="C7" s="8">
-        <f>C5*12</f>
-        <v>357732000.0</v>
-      </c>
-      <c r="D7" s="9">
-        <f>C7-B7</f>
-        <v>-178668000.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reduccion de costo</t>
-        </is>
-      </c>
-      <c r="D8" s="10">
-        <f>(B5-C5)/B5</f>
-        <v>0.33308724832214764</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DESGLOSE FLOTA ELECTRICA (CLP/mes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Leasing electrico</t>
-        </is>
-      </c>
-      <c r="B11" s="8">
-        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)</f>
-        <v>9520000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Energia electrica</t>
-        </is>
-      </c>
-      <c r="B12" s="8">
-        <f>(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)</f>
-        <v>1125000.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Infraestructura de carga</t>
-        </is>
-      </c>
-      <c r="B13" s="8">
-        <f>(Supuestos!$B$10*Supuestos!$B$24)</f>
-        <v>175000</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Conductores + peonetas</t>
-        </is>
-      </c>
-      <c r="B14" s="8">
-        <f>(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))</f>
-        <v>14280000.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sobrekilometraje</t>
-        </is>
-      </c>
-      <c r="B15" s="8">
-        <f>(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)</f>
-        <v>1350000</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Multas / deducibles</t>
-        </is>
-      </c>
-      <c r="B16" s="8">
-        <f>Supuestos!$B$29</f>
-        <v>500000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overhead de flota</t>
-        </is>
-      </c>
-      <c r="B17" s="8">
-        <f>(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)</f>
-        <v>2861000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TOTAL</t>
-        </is>
-      </c>
-      <c r="B18" s="9">
-        <f>SUM(B11:B17)</f>
-        <v>29811000.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">METRICAS DE DECISION</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ahorro / mes</t>
-        </is>
-      </c>
-      <c r="B21" s="8">
-        <f>B5-C5</f>
-        <v>14889000.0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ahorro / ano</t>
-        </is>
-      </c>
-      <c r="B22" s="8">
-        <f>(B5-C5)*12</f>
-        <v>178668000.0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ahorro 3 anos (nominal)</t>
-        </is>
-      </c>
-      <c r="B23" s="8">
-        <f>(B5-C5)*36</f>
-        <v>536004000.0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Punto de equilibrio (envios/mes)</t>
-        </is>
-      </c>
-      <c r="B24" s="11">
-        <f>C5/Supuestos!$B$8</f>
-        <v>10003.691275167785</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capacidad de la flota (envios/mes)</t>
-        </is>
-      </c>
-      <c r="B25" s="11">
-        <f>Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10</f>
-        <v>18480</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Utilizacion actual</t>
-        </is>
-      </c>
-      <c r="B26" s="10">
-        <f>Supuestos!$B$5/(Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10)</f>
-        <v>0.8116883116883117</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Holgura para crecer (envios/mes)</t>
-        </is>
-      </c>
-      <c r="B27" s="11">
-        <f>Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10-Supuestos!$B$5</f>
-        <v>3480</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
@@ -1129,301 +1125,288 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">TARIFA COMO OPERADOR LOGISTICO  (margen objetivo sobre venta)</t>
+          <t xml:space="preserve">EVALUACION: FLOTA ELECTRICA vs COURIER</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarifa que debes cobrar para cubrir costos y dejar el margen de Supuestos!B41. Compara contra el courier ($/envio actual).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Margen objetivo:</t>
-        </is>
-      </c>
-      <c r="B3" s="10">
-        <f>Supuestos!$B$41</f>
-        <v>0.3</v>
+          <t xml:space="preserve">Moviles del escenario base (editar en Supuestos!B10):</t>
+        </is>
+      </c>
+      <c r="B2" s="11">
+        <f>Supuestos!$B$10</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concepto</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Courier</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flota Electrica</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diferencia</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Concepto</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Flota Electrica</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Flota Petrolera</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Courier (ref.)</t>
-        </is>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo total / mes</t>
+        </is>
+      </c>
+      <c r="B5" s="8">
+        <f>Supuestos!$B$8*Supuestos!$B$5</f>
+        <v>44700000</v>
+      </c>
+      <c r="C5" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+(Supuestos!$B$10*Supuestos!$B$24)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
+        <v>29811000.0</v>
+      </c>
+      <c r="D5" s="9">
+        <f>C5-B5</f>
+        <v>-14889000.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Costo total / mes</t>
+          <t xml:space="preserve">Costo por envio</t>
         </is>
       </c>
       <c r="B6" s="8">
-        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+(Supuestos!$B$10*Supuestos!$B$24)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
-        <v>29811000.0</v>
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
       </c>
       <c r="C6" s="8">
-        <f>(Supuestos!$B$10*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
-        <v>29701000.0</v>
-      </c>
-      <c r="D6" s="8">
-        <f>Supuestos!$B$8*Supuestos!$B$5</f>
-        <v>44700000</v>
+        <f>C5/Supuestos!$B$5</f>
+        <v>1987.4</v>
+      </c>
+      <c r="D6" s="9">
+        <f>C6-B6</f>
+        <v>-992.5999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Costo por envio</t>
+          <t xml:space="preserve">Costo total / ano</t>
         </is>
       </c>
       <c r="B7" s="8">
-        <f>B6/Supuestos!$B$5</f>
-        <v>1987.4</v>
+        <f>B5*12</f>
+        <v>536400000</v>
       </c>
       <c r="C7" s="8">
-        <f>C6/Supuestos!$B$5</f>
-        <v>1980.0666666666666</v>
-      </c>
-      <c r="D7" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
+        <f>C5*12</f>
+        <v>357732000.0</v>
+      </c>
+      <c r="D7" s="9">
+        <f>C7-B7</f>
+        <v>-178668000.0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TARIFA por envio (con margen)</t>
-        </is>
-      </c>
-      <c r="B8" s="9">
-        <f>B7/(1-Supuestos!$B$41)</f>
-        <v>2839.1428571428573</v>
-      </c>
-      <c r="C8" s="9">
-        <f>C7/(1-Supuestos!$B$41)</f>
-        <v>2828.666666666667</v>
-      </c>
-      <c r="D8" s="9">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Facturacion / mes (a esa tarifa)</t>
-        </is>
-      </c>
-      <c r="B9" s="8">
-        <f>B6/(1-Supuestos!$B$41)</f>
-        <v>42587142.85714286</v>
-      </c>
-      <c r="C9" s="8">
-        <f>C6/(1-Supuestos!$B$41)</f>
-        <v>42430000.0</v>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reduccion de costo</t>
+        </is>
+      </c>
+      <c r="D8" s="10">
+        <f>(B5-C5)/B5</f>
+        <v>0.33308724832214764</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Margen $ / mes</t>
-        </is>
-      </c>
-      <c r="B10" s="8">
-        <f>B9-B6</f>
-        <v>12776142.857142858</v>
-      </c>
-      <c r="C10" s="8">
-        <f>C9-C6</f>
-        <v>12729000.0</v>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DESGLOSE FLOTA ELECTRICA (CLP/mes)</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Margen $ / ano</t>
-        </is>
-      </c>
-      <c r="B11" s="9">
-        <f>B10*12</f>
-        <v>153313714.2857143</v>
-      </c>
-      <c r="C11" s="9">
-        <f>C10*12</f>
-        <v>152748000.0</v>
+          <t xml:space="preserve">Leasing electrico</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)</f>
+        <v>9520000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarifa vs courier (ahorro/envio)</t>
-        </is>
-      </c>
-      <c r="B12" s="9">
-        <f>Supuestos!$B$8-B8</f>
-        <v>140.85714285714266</v>
-      </c>
-      <c r="C12" s="9">
-        <f>Supuestos!$B$8-C8</f>
-        <v>151.33333333333303</v>
+          <t xml:space="preserve">Energia electrica</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)</f>
+        <v>1125000.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tarifa % bajo el courier</t>
-        </is>
-      </c>
-      <c r="B13" s="10">
-        <f>(Supuestos!$B$8-B8)/Supuestos!$B$8</f>
-        <v>0.04726749760306801</v>
-      </c>
-      <c r="C13" s="10">
-        <f>(Supuestos!$B$8-C8)/Supuestos!$B$8</f>
-        <v>0.050782997762863435</v>
+          <t xml:space="preserve">Infraestructura de carga</t>
+        </is>
+      </c>
+      <c r="B13" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$24)</f>
+        <v>175000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conductores + peonetas</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))</f>
+        <v>14280000.0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TARIFA POR ENVIO SEGUN TAMANO DE FLOTA (con margen objetivo)</t>
-        </is>
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sobrekilometraje</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)</f>
+        <v>1350000</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Moviles (N)</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarifa Elec.</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarifa Pet.</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Courier (ref.)</t>
-        </is>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Multas / deducibles</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>Supuestos!$B$29</f>
+        <v>500000</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11">
-        <v>10</v>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overhead de flota</t>
+        </is>
       </c>
       <c r="B17" s="8">
-        <f>(($A17*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A17*Supuestos!$B$24)+($A17*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A17*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A17*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>3692.857142857143</v>
-      </c>
-      <c r="C17" s="8">
-        <f>(($A17*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A17*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A17*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A17*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>3595.2380952380954</v>
-      </c>
-      <c r="D17" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
+        <f>(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)</f>
+        <v>2861000</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11">
-        <v>9</v>
-      </c>
-      <c r="B18" s="8">
-        <f>(($A18*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A18*Supuestos!$B$24)+($A18*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A18*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A18*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>3408.2857142857147</v>
-      </c>
-      <c r="C18" s="8">
-        <f>(($A18*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A18*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A18*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A18*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>3339.7142857142862</v>
-      </c>
-      <c r="D18" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11">
-        <v>8</v>
-      </c>
-      <c r="B19" s="8">
-        <f>(($A19*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A19*Supuestos!$B$24)+($A19*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A19*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A19*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>3123.714285714286</v>
-      </c>
-      <c r="C19" s="8">
-        <f>(($A19*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A19*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A19*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A19*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>3084.1904761904766</v>
-      </c>
-      <c r="D19" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="9">
+        <f>SUM(B11:B17)</f>
+        <v>29811000.0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11">
-        <v>7</v>
-      </c>
-      <c r="B20" s="8">
-        <f>(($A20*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A20*Supuestos!$B$24)+($A20*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A20*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A20*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>2839.1428571428573</v>
-      </c>
-      <c r="C20" s="8">
-        <f>(($A20*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A20*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A20*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A20*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>2828.666666666667</v>
-      </c>
-      <c r="D20" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">METRICAS DE DECISION</t>
+        </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11">
-        <v>6</v>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahorro / mes</t>
+        </is>
       </c>
       <c r="B21" s="8">
-        <f>(($A21*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A21*Supuestos!$B$24)+($A21*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A21*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A21*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>2554.571428571429</v>
-      </c>
-      <c r="C21" s="8">
-        <f>(($A21*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A21*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A21*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A21*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
-        <v>2573.1428571428573</v>
-      </c>
-      <c r="D21" s="8">
-        <f>Supuestos!$B$8</f>
-        <v>2980</v>
+        <f>B5-C5</f>
+        <v>14889000.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahorro / ano</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>(B5-C5)*12</f>
+        <v>178668000.0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nota: margen sobre venta -&gt; tarifa = costo / (1 - margen). Si la tarifa es menor al courier, eres competitivo Y rentable.</t>
-        </is>
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ahorro 3 anos (nominal)</t>
+        </is>
+      </c>
+      <c r="B23" s="8">
+        <f>(B5-C5)*36</f>
+        <v>536004000.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Punto de equilibrio (envios/mes)</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>C5/Supuestos!$B$8</f>
+        <v>10003.691275167785</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capacidad de la flota (envios/mes)</t>
+        </is>
+      </c>
+      <c r="B25" s="11">
+        <f>Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10</f>
+        <v>18480</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utilizacion actual</t>
+        </is>
+      </c>
+      <c r="B26" s="10">
+        <f>Supuestos!$B$5/(Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10)</f>
+        <v>0.8116883116883117</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Holgura para crecer (envios/mes)</t>
+        </is>
+      </c>
+      <c r="B27" s="11">
+        <f>Supuestos!$B$7*Supuestos!$B$6*Supuestos!$B$10-Supuestos!$B$5</f>
+        <v>3480</v>
       </c>
     </row>
   </sheetData>
@@ -1431,6 +1414,319 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA COMO OPERADOR LOGISTICO  (margen objetivo sobre venta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa que debes cobrar para cubrir costos y dejar el margen de Supuestos!B41. Compara contra el courier ($/envio actual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen objetivo:</t>
+        </is>
+      </c>
+      <c r="B3" s="10">
+        <f>Supuestos!$B$41</f>
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concepto</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flota Electrica</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flota Petrolera</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Courier (ref.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo total / mes</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+(Supuestos!$B$10*Supuestos!$B$24)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
+        <v>29811000.0</v>
+      </c>
+      <c r="C6" s="8">
+        <f>(Supuestos!$B$10*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+(Supuestos!$B$10*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+Supuestos!$B$10*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-Supuestos!$B$10*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29</f>
+        <v>29701000.0</v>
+      </c>
+      <c r="D6" s="8">
+        <f>Supuestos!$B$8*Supuestos!$B$5</f>
+        <v>44700000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costo por envio</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>B6/Supuestos!$B$5</f>
+        <v>1987.4</v>
+      </c>
+      <c r="C7" s="8">
+        <f>C6/Supuestos!$B$5</f>
+        <v>1980.0666666666666</v>
+      </c>
+      <c r="D7" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA por envio (con margen)</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>B7/(1-Supuestos!$B$41)</f>
+        <v>2839.1428571428573</v>
+      </c>
+      <c r="C8" s="9">
+        <f>C7/(1-Supuestos!$B$41)</f>
+        <v>2828.666666666667</v>
+      </c>
+      <c r="D8" s="9">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facturacion / mes (a esa tarifa)</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>B6/(1-Supuestos!$B$41)</f>
+        <v>42587142.85714286</v>
+      </c>
+      <c r="C9" s="8">
+        <f>C6/(1-Supuestos!$B$41)</f>
+        <v>42430000.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen $ / mes</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>B9-B6</f>
+        <v>12776142.857142858</v>
+      </c>
+      <c r="C10" s="8">
+        <f>C9-C6</f>
+        <v>12729000.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Margen $ / ano</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>B10*12</f>
+        <v>153313714.2857143</v>
+      </c>
+      <c r="C11" s="9">
+        <f>C10*12</f>
+        <v>152748000.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa vs courier (ahorro/envio)</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>Supuestos!$B$8-B8</f>
+        <v>140.85714285714266</v>
+      </c>
+      <c r="C12" s="9">
+        <f>Supuestos!$B$8-C8</f>
+        <v>151.33333333333303</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa % bajo el courier</t>
+        </is>
+      </c>
+      <c r="B13" s="10">
+        <f>(Supuestos!$B$8-B8)/Supuestos!$B$8</f>
+        <v>0.04726749760306801</v>
+      </c>
+      <c r="C13" s="10">
+        <f>(Supuestos!$B$8-C8)/Supuestos!$B$8</f>
+        <v>0.050782997762863435</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARIFA POR ENVIO SEGUN TAMANO DE FLOTA (con margen objetivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moviles (N)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa Elec.</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarifa Pet.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Courier (ref.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11">
+        <v>10</v>
+      </c>
+      <c r="B17" s="8">
+        <f>(($A17*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A17*Supuestos!$B$24)+($A17*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A17*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A17*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3692.857142857143</v>
+      </c>
+      <c r="C17" s="8">
+        <f>(($A17*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A17*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A17*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A17*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3595.2380952380954</v>
+      </c>
+      <c r="D17" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11">
+        <v>9</v>
+      </c>
+      <c r="B18" s="8">
+        <f>(($A18*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A18*Supuestos!$B$24)+($A18*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A18*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A18*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3408.2857142857147</v>
+      </c>
+      <c r="C18" s="8">
+        <f>(($A18*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A18*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A18*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A18*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3339.7142857142862</v>
+      </c>
+      <c r="D18" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11">
+        <v>8</v>
+      </c>
+      <c r="B19" s="8">
+        <f>(($A19*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A19*Supuestos!$B$24)+($A19*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A19*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A19*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3123.714285714286</v>
+      </c>
+      <c r="C19" s="8">
+        <f>(($A19*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A19*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A19*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A19*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>3084.1904761904766</v>
+      </c>
+      <c r="D19" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11">
+        <v>7</v>
+      </c>
+      <c r="B20" s="8">
+        <f>(($A20*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A20*Supuestos!$B$24)+($A20*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A20*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A20*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2839.1428571428573</v>
+      </c>
+      <c r="C20" s="8">
+        <f>(($A20*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A20*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A20*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A20*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2828.666666666667</v>
+      </c>
+      <c r="D20" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11">
+        <v>6</v>
+      </c>
+      <c r="B21" s="8">
+        <f>(($A21*Supuestos!$B$18*Supuestos!$B$9)+(Supuestos!$B$13*Supuestos!$B$21*Supuestos!$B$20)+($A21*Supuestos!$B$24)+($A21*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A21*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A21*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2554.571428571429</v>
+      </c>
+      <c r="C21" s="8">
+        <f>(($A21*Supuestos!$B$19*Supuestos!$B$9)+(Supuestos!$B$13/Supuestos!$B$23*Supuestos!$B$22)+($A21*Supuestos!$B$27*(2-Supuestos!$B$28))+(Supuestos!$B$30+$A21*Supuestos!$B$31)+(MAX(0,Supuestos!$B$13-$A21*Supuestos!$B$14)*Supuestos!$B$15)+Supuestos!$B$29)/Supuestos!$B$5/(1-Supuestos!$B$41)</f>
+        <v>2573.1428571428573</v>
+      </c>
+      <c r="D21" s="8">
+        <f>Supuestos!$B$8</f>
+        <v>2980</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nota: margen sobre venta -&gt; tarifa = costo / (1 - margen). Si la tarifa es menor al courier, eres competitivo Y rentable.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>

</xml_diff>